<commit_message>
se termina metodo de exportacion de directosio
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/plantilla_directorio.xlsx
+++ b/imagenes_guardadas/plantilla_directorio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\acrivera-sis\imagenes_guardadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05B63F5-3B4D-4466-AC18-22E2029FD6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EEC95A7-4357-483B-8DDF-8BFFAB2F4C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{87150DB9-E01B-4AEC-9ADF-5D7D3FBAF6A1}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="ACR" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ACR!$B$5:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ACR!$B$5:$E$5</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>PURGA</t>
   </si>
@@ -61,12 +61,6 @@
   </si>
   <si>
     <t>Extensión</t>
-  </si>
-  <si>
-    <t>20/01/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -277,11 +271,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -705,112 +696,81 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="38" style="8" customWidth="1"/>
-    <col min="3" max="3" width="36.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="42" style="8" customWidth="1"/>
-    <col min="5" max="5" width="22.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="33.140625" style="4" customWidth="1"/>
-    <col min="8" max="10" width="11.42578125" style="4"/>
-    <col min="11" max="11" width="11.85546875" style="4" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" style="4"/>
-    <col min="13" max="13" width="12.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="11.42578125" style="4"/>
-    <col min="16" max="16" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="11.42578125" style="4"/>
+    <col min="1" max="1" width="3.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="38" style="7" customWidth="1"/>
+    <col min="3" max="3" width="36.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42" style="7" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="33.140625" style="3" customWidth="1"/>
+    <col min="8" max="10" width="11.42578125" style="3"/>
+    <col min="11" max="11" width="11.85546875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" style="3"/>
+    <col min="13" max="13" width="12.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="11.42578125" style="3"/>
+    <col min="16" max="16" width="11.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="K1" s="16" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="K1" s="15" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" ht="18.75" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="17" t="s">
+    <row r="2" spans="1:11" s="1" customFormat="1" ht="18.75" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="3"/>
-      <c r="K2" s="9"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="2"/>
+      <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:11" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.35">
-      <c r="A3" s="3"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="6" t="s">
+    <row r="3" spans="1:11" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.35">
+      <c r="A3" s="2"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="K3" s="9"/>
+      <c r="F3" s="2"/>
+      <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:11" s="2" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="3"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="3"/>
-      <c r="K4" s="15"/>
+    <row r="4" spans="1:11" s="1" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="2"/>
+      <c r="K4" s="14"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D6" s="1"/>
-      <c r="K6" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D7" s="1"/>
-      <c r="K7" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D8" s="1"/>
-      <c r="K8" s="8"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D9" s="1"/>
-      <c r="G9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D10" s="1"/>
-      <c r="K10" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="B5:E10" xr:uid="{D86A5473-DB2B-4115-A887-AC4943C8BE85}"/>
+  <autoFilter ref="B5:E5" xr:uid="{D86A5473-DB2B-4115-A887-AC4943C8BE85}"/>
   <mergeCells count="1">
     <mergeCell ref="C2:D4"/>
   </mergeCells>
@@ -822,6 +782,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <DueDate xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
+    <Grade xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
+    <Quarter xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
+    <AssignedDate xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
+    <Teacher xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Teacher>
+    <Description xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DD6562627BE4DD48869B7C063DC1C002" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="dc475340b07e0068f10667b9462b67b2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fee71d3c-8b14-4e13-9a47-aa074b04d610" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="981e5bd1d6bd900e7e06cefd7e1d4026" ns2:_="">
     <xsd:import namespace="fee71d3c-8b14-4e13-9a47-aa074b04d610"/>
@@ -1027,35 +1015,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B427448-C403-4BE3-988C-153D28238C33}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fee71d3c-8b14-4e13-9a47-aa074b04d610"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <DueDate xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
-    <Grade xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
-    <Quarter xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
-    <AssignedDate xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
-    <Teacher xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Teacher>
-    <Description xmlns="fee71d3c-8b14-4e13-9a47-aa074b04d610" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08E00009-83E5-4D30-9694-E7BFE88F31D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A66C09C9-BD88-4506-ABE8-81DF5FDB1C26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1071,22 +1049,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08E00009-83E5-4D30-9694-E7BFE88F31D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B427448-C403-4BE3-988C-153D28238C33}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fee71d3c-8b14-4e13-9a47-aa074b04d610"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>